<commit_message>
Atualizações para 2aRQ 2026-2030
</commit_message>
<xml_diff>
--- a/inst/dados_premissas/2025/crescimento_mercado.xlsx
+++ b/inst/dados_premissas/2025/crescimento_mercado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Geracao Distribuida\PDE\PLAN26-30_1RQ\dados_premissas\2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Geracao Distribuida\PDE\PLAN26-30_2RQ\dados_premissas\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52AD1A9A-288D-46D9-AE65-051194B5212E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78FA7572-E9BB-47CD-838E-BC1339E3705D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -534,7 +534,7 @@
         <v>2026</v>
       </c>
       <c r="B18">
-        <v>0.02</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="4"/>
@@ -544,7 +544,7 @@
         <v>2027</v>
       </c>
       <c r="B19">
-        <v>2.4E-2</v>
+        <v>0.02</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="4"/>

</xml_diff>